<commit_message>
Job tracker update 2026-10-08
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,116 +482,486 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>shifttechnology</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>QA Engineer Intern (6 months)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>React, TypeScript, Docker, Kubernetes</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>shifttechnology</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Full stack Engineer Intern (6 months)</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Java, React</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>orderbird GmbH</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Berlin</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Head of Software Engineering (d/f/m)</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Design System Director (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
         <is>
           <t>Arbeitnow</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G14" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G4"/>
+  <autoFilter ref="A1:G14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-09
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$20</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,34 +492,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,27 +529,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -566,27 +566,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -603,27 +603,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -640,7 +640,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -650,17 +650,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -677,27 +677,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -714,27 +714,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -751,27 +751,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -788,27 +788,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -825,27 +825,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -872,17 +872,17 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -894,32 +894,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -936,27 +936,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
@@ -968,106 +968,106 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>autoscout24</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
         </is>
       </c>
     </row>
@@ -1079,37 +1079,111 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D20" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
+      <c r="G20" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G18"/>
+  <autoFilter ref="A1:G20"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-10
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,34 +492,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,34 +529,34 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -566,34 +566,34 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,34 +603,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,27 +640,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -677,27 +677,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -714,17 +714,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -751,27 +751,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -788,27 +788,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -825,27 +825,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -862,27 +862,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -899,27 +899,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -936,27 +936,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -968,32 +968,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -1010,27 +1010,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -1047,34 +1047,34 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,106 +1084,217 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr">
+      <c r="G23" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G20"/>
+  <autoFilter ref="A1:G23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-11
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$25</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,34 +492,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,27 +529,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
@@ -566,34 +566,34 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,34 +603,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,34 +640,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -677,34 +677,34 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,27 +714,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -751,27 +751,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -788,27 +788,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -825,7 +825,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -835,17 +835,17 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -862,27 +862,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -899,27 +899,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -936,27 +936,27 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -973,27 +973,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -1010,27 +1010,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -1057,17 +1057,17 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -1079,32 +1079,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -1121,27 +1121,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
@@ -1153,106 +1153,106 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>autoscout24</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
         </is>
       </c>
     </row>
@@ -1264,37 +1264,111 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G25" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G23"/>
+  <autoFilter ref="A1:G25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-12
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$32</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,118 +482,118 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,34 +603,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,7 +640,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -650,61 +650,61 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,34 +714,34 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -751,34 +751,34 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -788,34 +788,34 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -825,17 +825,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -845,14 +845,14 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -862,34 +862,34 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -899,34 +899,34 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -936,7 +936,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -946,24 +946,24 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -973,27 +973,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -1010,27 +1010,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -1047,27 +1047,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -1084,27 +1084,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -1121,27 +1121,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -1153,32 +1153,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -1195,27 +1195,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -1232,143 +1232,402 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Design System Director (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr">
+      <c r="D32" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr">
+      <c r="E32" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
+      <c r="F32" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr">
+      <c r="G32" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G25"/>
+  <autoFilter ref="A1:G32"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-13
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$32</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,44 +482,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -539,61 +539,61 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,17 +603,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -623,14 +623,14 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,17 +640,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -660,44 +660,44 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -709,113 +709,113 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -825,34 +825,34 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -862,71 +862,71 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -936,34 +936,34 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -973,34 +973,34 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1010,34 +1010,34 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1047,34 +1047,34 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,34 +1084,34 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1121,34 +1121,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1158,34 +1158,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,27 +1195,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -1232,27 +1232,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -1269,27 +1269,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -1306,27 +1306,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -1343,27 +1343,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -1380,27 +1380,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -1412,32 +1412,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -1454,27 +1454,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -1491,143 +1491,365 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Design System Director (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C32" t="inlineStr">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr">
+      <c r="D38" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E32" t="inlineStr">
+      <c r="E38" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F32" t="inlineStr">
+      <c r="F38" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr">
+      <c r="G38" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G32"/>
+  <autoFilter ref="A1:G38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-14
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$45</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,108 +492,108 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,34 +603,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,34 +640,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -677,108 +677,108 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -788,34 +788,34 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -825,34 +825,34 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -862,17 +862,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -882,51 +882,51 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -936,145 +936,145 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,34 +1084,34 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1131,61 +1131,61 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,34 +1195,34 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1232,34 +1232,34 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1269,34 +1269,34 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1306,17 +1306,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1326,14 +1326,14 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1343,34 +1343,34 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1380,34 +1380,34 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1427,24 +1427,24 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1454,27 +1454,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -1491,27 +1491,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -1528,27 +1528,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -1565,27 +1565,27 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -1602,27 +1602,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -1634,32 +1634,32 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -1676,27 +1676,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -1713,143 +1713,402 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Design System Director (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C38" t="inlineStr">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr">
+      <c r="D45" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr">
+      <c r="E45" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F38" t="inlineStr">
+      <c r="F45" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr">
+      <c r="G45" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G38"/>
+  <autoFilter ref="A1:G45"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-15
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$45</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$51</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G45"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,34 +492,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,71 +529,71 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,34 +603,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,34 +640,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -677,27 +677,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -714,34 +714,34 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -751,34 +751,34 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -788,34 +788,34 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -825,34 +825,34 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -862,34 +862,34 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -899,34 +899,34 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -936,71 +936,71 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1020,61 +1020,61 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,17 +1084,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1104,14 +1104,14 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1121,17 +1121,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -1141,44 +1141,44 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -1190,113 +1190,113 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1306,34 +1306,34 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1343,71 +1343,71 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1417,34 +1417,34 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1454,34 +1454,34 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1491,34 +1491,34 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1528,34 +1528,34 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1565,34 +1565,34 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1602,34 +1602,34 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1639,34 +1639,34 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1676,27 +1676,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -1713,27 +1713,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -1750,27 +1750,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -1787,27 +1787,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -1824,27 +1824,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -1861,27 +1861,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -1893,32 +1893,32 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -1935,27 +1935,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -1972,143 +1972,365 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Design System Director (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D51" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E51" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F51" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G51" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G45"/>
+  <autoFilter ref="A1:G51"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-16
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$51</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$53</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,34 +492,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,27 +529,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -566,27 +566,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
@@ -603,27 +603,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
@@ -640,27 +640,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
@@ -677,34 +677,34 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,34 +714,34 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -751,27 +751,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -783,32 +783,32 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -825,27 +825,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
@@ -857,32 +857,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
@@ -899,27 +899,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
@@ -936,34 +936,34 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -973,64 +973,64 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -1047,27 +1047,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
@@ -1079,32 +1079,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
@@ -1121,27 +1121,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
@@ -1158,101 +1158,101 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -1269,27 +1269,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -1301,32 +1301,32 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
@@ -1338,32 +1338,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
@@ -1375,32 +1375,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
@@ -1417,71 +1417,71 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1491,34 +1491,34 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1528,34 +1528,34 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1565,27 +1565,27 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
@@ -1602,34 +1602,34 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1639,34 +1639,34 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1676,34 +1676,34 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1713,34 +1713,34 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1750,27 +1750,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -1787,27 +1787,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -1824,27 +1824,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1861,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1871,17 +1871,17 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -1898,27 +1898,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -1935,27 +1935,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -1972,27 +1972,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -2009,27 +2009,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -2046,27 +2046,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -2093,17 +2093,17 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -2115,32 +2115,32 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -2157,27 +2157,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
@@ -2189,106 +2189,106 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>autoscout24</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
         </is>
       </c>
     </row>
@@ -2300,37 +2300,111 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D53" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E53" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F53" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G53" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G51"/>
+  <autoFilter ref="A1:G53"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-17
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$54</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G53"/>
+  <dimension ref="A1:G54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,27 +492,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
@@ -529,34 +529,34 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -566,27 +566,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -603,27 +603,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
@@ -650,17 +650,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
@@ -677,27 +677,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
@@ -714,27 +714,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
@@ -751,34 +751,34 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -788,27 +788,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -825,27 +825,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -857,32 +857,32 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
@@ -894,32 +894,32 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
@@ -946,17 +946,17 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
@@ -973,27 +973,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
@@ -1015,29 +1015,29 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1047,27 +1047,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -1079,32 +1079,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
@@ -1116,32 +1116,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
@@ -1168,17 +1168,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
@@ -1195,17 +1195,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
@@ -1232,64 +1232,64 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -1306,27 +1306,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -1343,27 +1343,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
@@ -1375,32 +1375,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
@@ -1449,32 +1449,32 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
@@ -1486,39 +1486,39 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1528,27 +1528,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
@@ -1565,34 +1565,34 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1602,27 +1602,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
@@ -1639,27 +1639,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
@@ -1676,34 +1676,34 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1713,27 +1713,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
@@ -1750,34 +1750,34 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1787,27 +1787,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -1834,17 +1834,17 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -1861,27 +1861,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -1898,7 +1898,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1908,17 +1908,17 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -1945,17 +1945,17 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -1972,27 +1972,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -2009,7 +2009,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2019,17 +2019,17 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -2046,27 +2046,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -2083,27 +2083,27 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -2130,17 +2130,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
@@ -2177,7 +2177,7 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -2189,32 +2189,32 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
@@ -2226,32 +2226,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
@@ -2268,64 +2268,64 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>autoscout24</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
         </is>
       </c>
     </row>
@@ -2342,27 +2342,27 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Sporty Group</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Frontend Engineering Team Lead - MarTech</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
         </is>
       </c>
     </row>
@@ -2374,37 +2374,74 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D54" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E54" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F54" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G54" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G53"/>
+  <autoFilter ref="A1:G54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-18
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,34 +492,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,34 +529,34 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -566,34 +566,34 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,34 +603,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,34 +640,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -677,34 +677,34 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,34 +714,34 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -751,71 +751,71 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -825,34 +825,34 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -862,71 +862,71 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -936,34 +936,34 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -973,34 +973,34 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1010,34 +1010,34 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1047,34 +1047,34 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,71 +1084,71 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1158,34 +1158,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,54 +1195,54 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1252,14 +1252,14 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1269,145 +1269,145 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1417,108 +1417,108 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1528,34 +1528,34 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1565,34 +1565,34 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1602,54 +1602,54 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -1659,88 +1659,88 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1750,17 +1750,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1770,14 +1770,14 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1787,71 +1787,71 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1861,34 +1861,34 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1898,7 +1898,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1908,24 +1908,24 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1935,34 +1935,34 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1972,34 +1972,34 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2009,34 +2009,34 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2046,34 +2046,34 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2083,34 +2083,34 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2120,27 +2120,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -2157,27 +2157,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -2194,27 +2194,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -2226,32 +2226,32 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -2268,27 +2268,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -2305,7 +2305,7 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -2315,133 +2315,466 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Hawkeyeinnovations</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Budapest, Hungary</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, Docker, AWS</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Design System Director (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D63" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E63" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F63" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G63" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G54"/>
+  <autoFilter ref="A1:G63"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-19
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,44 +482,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,64 +529,64 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -603,27 +603,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -640,27 +640,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -677,27 +677,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -714,27 +714,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
@@ -751,27 +751,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
@@ -783,39 +783,39 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -825,34 +825,34 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -862,71 +862,71 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -936,34 +936,34 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -973,12 +973,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -993,14 +993,14 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1010,27 +1010,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -1047,27 +1047,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
@@ -1084,27 +1084,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
@@ -1121,34 +1121,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1158,34 +1158,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,64 +1195,64 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -1269,27 +1269,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -1306,27 +1306,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
@@ -1338,32 +1338,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
@@ -1380,34 +1380,34 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1417,71 +1417,71 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1491,27 +1491,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -1528,27 +1528,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
@@ -1560,32 +1560,32 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
@@ -1602,138 +1602,138 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -1745,32 +1745,32 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -1782,32 +1782,32 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
@@ -1824,27 +1824,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
@@ -1861,34 +1861,34 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1898,71 +1898,71 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1972,34 +1972,34 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2009,34 +2009,34 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2046,34 +2046,34 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2083,34 +2083,34 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2120,34 +2120,34 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2157,34 +2157,34 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2194,34 +2194,34 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2231,27 +2231,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -2268,27 +2268,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -2305,17 +2305,17 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
@@ -2325,7 +2325,7 @@
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -2342,27 +2342,27 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -2379,27 +2379,27 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -2416,27 +2416,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -2453,27 +2453,27 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -2490,27 +2490,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -2527,27 +2527,27 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -2559,32 +2559,32 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -2601,27 +2601,27 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -2638,34 +2638,34 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2675,106 +2675,217 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D66" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E66" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F66" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
+      <c r="G66" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G63"/>
+  <autoFilter ref="A1:G66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-20
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$70</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G66"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,118 +482,118 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,71 +603,71 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -677,64 +677,64 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -751,27 +751,27 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -788,27 +788,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -825,27 +825,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -862,27 +862,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
@@ -894,39 +894,39 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -936,34 +936,34 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -973,34 +973,34 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1010,71 +1010,71 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,34 +1084,34 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1121,34 +1121,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1158,27 +1158,27 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -1195,27 +1195,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
@@ -1232,34 +1232,34 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1269,34 +1269,34 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1306,71 +1306,71 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1380,27 +1380,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -1417,27 +1417,27 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -1454,27 +1454,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
@@ -1486,39 +1486,39 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1528,12 +1528,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1548,51 +1548,51 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1602,34 +1602,34 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1639,27 +1639,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -1676,27 +1676,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
@@ -1708,150 +1708,150 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1861,27 +1861,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -1893,32 +1893,32 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -1935,27 +1935,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
@@ -1967,39 +1967,39 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2009,34 +2009,34 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2046,71 +2046,71 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2120,34 +2120,34 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2157,34 +2157,34 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2194,34 +2194,34 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2231,7 +2231,7 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -2241,24 +2241,24 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2268,34 +2268,34 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2305,34 +2305,34 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2342,34 +2342,34 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2379,27 +2379,27 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -2416,27 +2416,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -2453,27 +2453,27 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -2490,27 +2490,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -2527,27 +2527,27 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -2564,27 +2564,27 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -2601,27 +2601,27 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -2638,27 +2638,27 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -2670,32 +2670,32 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -2712,27 +2712,27 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -2749,71 +2749,71 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2823,69 +2823,217 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D66" t="inlineStr">
+      <c r="D70" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E66" t="inlineStr">
+      <c r="E70" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F70" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G66" t="inlineStr">
+      <c r="G70" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G66"/>
+  <autoFilter ref="A1:G70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-21
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,27 +492,27 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
@@ -524,32 +524,32 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
@@ -561,32 +561,32 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
@@ -603,64 +603,64 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
@@ -672,32 +672,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
@@ -709,69 +709,69 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -798,17 +798,17 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -825,27 +825,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -862,27 +862,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -899,27 +899,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
@@ -936,17 +936,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
@@ -973,27 +973,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
@@ -1020,7 +1020,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
@@ -1042,76 +1042,76 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1121,27 +1121,27 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
@@ -1158,34 +1158,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,27 +1195,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -1232,27 +1232,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
@@ -1279,17 +1279,17 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
@@ -1306,27 +1306,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
@@ -1343,27 +1343,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
@@ -1380,34 +1380,34 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1417,27 +1417,27 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -1454,27 +1454,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -1486,32 +1486,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
@@ -1523,32 +1523,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
@@ -1575,17 +1575,17 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
@@ -1602,27 +1602,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
@@ -1644,29 +1644,29 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1676,27 +1676,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -1708,32 +1708,32 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
@@ -1745,32 +1745,32 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
@@ -1797,17 +1797,17 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
@@ -1824,17 +1824,17 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
@@ -1861,64 +1861,64 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -1935,27 +1935,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -1972,27 +1972,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
@@ -2004,32 +2004,32 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2056,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
@@ -2078,32 +2078,32 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
@@ -2115,39 +2115,39 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2157,27 +2157,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
@@ -2194,34 +2194,34 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2231,27 +2231,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
@@ -2268,27 +2268,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
@@ -2305,34 +2305,34 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2342,27 +2342,27 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
@@ -2379,34 +2379,34 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2416,27 +2416,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -2463,17 +2463,17 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -2490,27 +2490,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -2527,7 +2527,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2537,17 +2537,17 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -2574,17 +2574,17 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -2601,27 +2601,27 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -2638,7 +2638,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2648,17 +2648,17 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -2675,27 +2675,27 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -2712,27 +2712,27 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -2759,17 +2759,17 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -2796,7 +2796,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -2818,32 +2818,32 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
@@ -2855,32 +2855,32 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
@@ -2897,64 +2897,64 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>autoscout24</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
         </is>
       </c>
     </row>
@@ -2971,27 +2971,27 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Sporty Group</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Frontend Engineering Team Lead - MarTech</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
         </is>
       </c>
     </row>
@@ -3003,37 +3003,74 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D70" t="inlineStr">
+      <c r="D71" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E70" t="inlineStr">
+      <c r="E71" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
+      <c r="G71" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G70"/>
+  <autoFilter ref="A1:G71"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-22
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$76</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G71"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,44 +482,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Coreweave</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Account Solution Architect</t>
+          <t>AI Software Engineer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
+          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,71 +529,71 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,34 +603,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>Principal Engineer (Software Engineering/Devops)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,71 +640,71 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>GradeMatch</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Eindhoven, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,34 +714,34 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -751,34 +751,34 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -788,34 +788,34 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -825,71 +825,71 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -899,64 +899,64 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -973,27 +973,27 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -1010,27 +1010,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -1047,27 +1047,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -1079,39 +1079,39 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1121,34 +1121,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1158,34 +1158,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,34 +1195,34 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1232,71 +1232,71 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1306,34 +1306,34 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1343,34 +1343,34 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1380,27 +1380,27 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -1417,34 +1417,34 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1454,34 +1454,34 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1491,71 +1491,71 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1565,34 +1565,34 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1602,27 +1602,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -1639,27 +1639,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -1676,108 +1676,108 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1787,34 +1787,34 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1824,34 +1824,34 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1861,27 +1861,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -1898,34 +1898,34 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1935,108 +1935,108 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2046,17 +2046,17 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
@@ -2066,14 +2066,14 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2083,27 +2083,27 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -2120,27 +2120,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -2152,76 +2152,76 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2231,34 +2231,34 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2268,71 +2268,71 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2342,34 +2342,34 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2379,34 +2379,34 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2416,34 +2416,34 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2453,34 +2453,34 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2490,34 +2490,34 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2527,34 +2527,34 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2564,34 +2564,34 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2601,27 +2601,27 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -2638,27 +2638,27 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -2675,27 +2675,27 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -2712,27 +2712,27 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -2749,27 +2749,27 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -2786,27 +2786,27 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -2823,27 +2823,27 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -2855,32 +2855,32 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -2897,27 +2897,27 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -2934,143 +2934,328 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D71" t="inlineStr">
+      <c r="D76" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E76" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F76" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G71" t="inlineStr">
+      <c r="G76" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G71"/>
+  <autoFilter ref="A1:G76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-23
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$84</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G76"/>
+  <dimension ref="A1:G84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,44 +482,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Breda, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>AI Software Engineer</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,34 +529,34 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Zoetermeer, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -566,34 +566,34 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
+          <t>Staff Engineer - Fullstack - Actions</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,71 +603,71 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Grip</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Principal Engineer (Software Engineering/Devops)</t>
+          <t>Join Our Talent Community: Solutions Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>GradeMatch</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Eindhoven, Noord-Brabant, Nederland</t>
+          <t>EMEA</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Full Stack Developer</t>
+          <t>Engineering Director - Commercial Systems</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
+          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -677,34 +677,34 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Coreweave</t>
+          <t>Banyansoftware</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Account Solution Architect</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -714,108 +714,108 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Staff Software Engineer, Payments</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Software Engineer, Payments Platform</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>AI Software Engineer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -825,7 +825,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -835,61 +835,61 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -899,71 +899,71 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Principal Engineer (Software Engineering/Devops)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>GradeMatch</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Eindhoven, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -973,34 +973,34 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1010,71 +1010,71 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,34 +1084,34 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1121,7 +1121,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1131,61 +1131,61 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,64 +1195,64 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -1264,39 +1264,39 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1306,34 +1306,34 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1343,34 +1343,34 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1380,34 +1380,34 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1417,34 +1417,34 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1454,34 +1454,34 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1491,34 +1491,34 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1528,71 +1528,71 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1602,34 +1602,34 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1639,34 +1639,34 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1676,71 +1676,71 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1750,34 +1750,34 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1787,34 +1787,34 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1824,34 +1824,34 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1861,34 +1861,34 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1898,71 +1898,71 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1972,54 +1972,54 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
@@ -2029,14 +2029,14 @@
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2046,34 +2046,34 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2083,182 +2083,182 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2268,71 +2268,71 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2342,34 +2342,34 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2379,145 +2379,145 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2527,7 +2527,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2537,24 +2537,24 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2564,17 +2564,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
@@ -2584,51 +2584,51 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2638,34 +2638,34 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2675,34 +2675,34 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2712,34 +2712,34 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2749,34 +2749,34 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2786,34 +2786,34 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2823,34 +2823,34 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2870,24 +2870,24 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2897,27 +2897,27 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -2934,27 +2934,27 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -2971,27 +2971,27 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -3008,27 +3008,27 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -3040,32 +3040,32 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -3082,27 +3082,27 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -3119,143 +3119,439 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>Design System Director (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D76" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr">
+      <c r="E84" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F76" t="inlineStr">
+      <c r="F84" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G76" t="inlineStr">
+      <c r="G84" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G76"/>
+  <autoFilter ref="A1:G84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-24
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$89</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G84"/>
+  <dimension ref="A1:G89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,34 +492,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Breda, Noord-Brabant, Nederland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
+          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,108 +529,108 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Zoetermeer, Zuid-Holland, Nederland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
+          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Staff Engineer - Fullstack - Actions</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
+          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Join Our Talent Community: Solutions Engineer</t>
+          <t>Software Engineering Director</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
+          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,27 +640,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Banyan Software</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EMEA</t>
+          <t>Belgium,  Germany,  Netherlands,  UK</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Engineering Director - Commercial Systems</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
+          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
         </is>
       </c>
     </row>
@@ -677,27 +677,27 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Banyansoftware</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Breda, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
         </is>
       </c>
     </row>
@@ -714,27 +714,27 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>Zoetermeer, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Staff Software Engineer, Payments</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
         </is>
       </c>
     </row>
@@ -751,108 +751,108 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Payments Platform</t>
+          <t>Staff Engineer - Fullstack - Actions</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>AI Software Engineer</t>
+          <t>Join Our Talent Community: Solutions Engineer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EMEA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
+          <t>Engineering Director - Commercial Systems</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
+          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -862,34 +862,34 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Banyansoftware</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -899,34 +899,34 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Grip</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Principal Engineer (Software Engineering/Devops)</t>
+          <t>Staff Software Engineer, Payments</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -936,71 +936,71 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GradeMatch</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Eindhoven, Noord-Brabant, Nederland</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Full Stack Developer</t>
+          <t>Senior Software Engineer, Payments Platform</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Coreweave</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Account Solution Architect</t>
+          <t>AI Software Engineer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
+          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1010,71 +1010,71 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,34 +1084,34 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>Principal Engineer (Software Engineering/Devops)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1121,71 +1121,71 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>GradeMatch</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Eindhoven, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,34 +1195,34 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1232,34 +1232,34 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1269,34 +1269,34 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1306,71 +1306,71 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1380,64 +1380,64 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -1454,27 +1454,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -1491,27 +1491,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -1528,27 +1528,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -1560,39 +1560,39 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1602,34 +1602,34 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1639,34 +1639,34 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1676,34 +1676,34 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1713,71 +1713,71 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1787,34 +1787,34 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1824,34 +1824,34 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1861,27 +1861,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -1898,34 +1898,34 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1935,34 +1935,34 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1972,71 +1972,71 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2046,34 +2046,34 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2083,27 +2083,27 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -2120,27 +2120,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -2157,108 +2157,108 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2268,34 +2268,34 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2305,34 +2305,34 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2342,27 +2342,27 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -2379,34 +2379,34 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2416,108 +2416,108 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2527,17 +2527,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -2547,14 +2547,14 @@
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2564,27 +2564,27 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -2601,27 +2601,27 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -2633,76 +2633,76 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2712,34 +2712,34 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2749,71 +2749,71 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2823,34 +2823,34 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2860,34 +2860,34 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2897,34 +2897,34 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2934,34 +2934,34 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2971,34 +2971,34 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3008,34 +3008,34 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3045,34 +3045,34 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3082,27 +3082,27 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -3119,27 +3119,27 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -3156,27 +3156,27 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -3193,27 +3193,27 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -3230,27 +3230,27 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -3267,27 +3267,27 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -3304,27 +3304,27 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -3336,32 +3336,32 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -3378,27 +3378,27 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -3415,143 +3415,328 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D84" t="inlineStr">
+      <c r="D89" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E84" t="inlineStr">
+      <c r="E89" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F84" t="inlineStr">
+      <c r="F89" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G84" t="inlineStr">
+      <c r="G89" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G84"/>
+  <autoFilter ref="A1:G89"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-25
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$89</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G89"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,111 +482,111 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Ireland,  Spain,  UK</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
+          <t>Presales Engineer (German Speaking)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
+          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Ireland,  UK</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
+          <t>Presales Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
+          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Malt</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
+          <t>Senior Engineering Manager - Payment</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
         </is>
       </c>
     </row>
@@ -598,32 +598,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Software Engineering Director</t>
+          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
         </is>
       </c>
     </row>
@@ -635,143 +635,143 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Banyan Software</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Belgium,  Germany,  Netherlands,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Breda, Noord-Brabant, Nederland</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
+          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Zoetermeer, Zuid-Holland, Nederland</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
+          <t>Software Engineering Director</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
+          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Banyan Software</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
+          <t>Belgium,  Germany,  Netherlands,  UK</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Staff Engineer - Fullstack - Actions</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
+          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
         </is>
       </c>
     </row>
@@ -788,27 +788,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
+          <t>Breda, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Join Our Talent Community: Solutions Engineer</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
         </is>
       </c>
     </row>
@@ -820,32 +820,32 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EMEA</t>
+          <t>Zoetermeer, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Engineering Director - Commercial Systems</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
         </is>
       </c>
     </row>
@@ -862,27 +862,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Banyansoftware</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Staff Engineer - Fullstack - Actions</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
         </is>
       </c>
     </row>
@@ -899,27 +899,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Staff Software Engineer, Payments</t>
+          <t>Join Our Talent Community: Solutions Engineer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
         </is>
       </c>
     </row>
@@ -931,76 +931,76 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>EMEA</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Payments Platform</t>
+          <t>Engineering Director - Commercial Systems</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
+          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Banyansoftware</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>AI Software Engineer</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1010,34 +1010,34 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
+          <t>Staff Software Engineer, Payments</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1047,27 +1047,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
+          <t>Senior Software Engineer, Payments Platform</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
         </is>
       </c>
     </row>
@@ -1079,32 +1079,32 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Grip</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Principal Engineer (Software Engineering/Devops)</t>
+          <t>AI Software Engineer</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
+          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
         </is>
       </c>
     </row>
@@ -1121,34 +1121,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GradeMatch</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Eindhoven, Noord-Brabant, Nederland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Full Stack Developer</t>
+          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript</t>
+          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1158,34 +1158,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Coreweave</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Account Solution Architect</t>
+          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,71 +1195,71 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Principal Engineer (Software Engineering/Devops)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>GradeMatch</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Eindhoven, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1269,27 +1269,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
@@ -1306,34 +1306,34 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1343,34 +1343,34 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1380,108 +1380,108 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1491,64 +1491,64 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -1565,27 +1565,27 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -1602,27 +1602,27 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -1639,27 +1639,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -1676,27 +1676,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
@@ -1713,27 +1713,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
@@ -1745,39 +1745,39 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1787,34 +1787,34 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1824,71 +1824,71 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1898,34 +1898,34 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1935,12 +1935,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1955,14 +1955,14 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1972,27 +1972,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -2009,27 +2009,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
@@ -2046,27 +2046,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
@@ -2083,34 +2083,34 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2120,34 +2120,34 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2157,64 +2157,64 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -2231,27 +2231,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -2268,27 +2268,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
@@ -2300,32 +2300,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
@@ -2342,34 +2342,34 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2379,71 +2379,71 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2453,27 +2453,27 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -2490,27 +2490,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
@@ -2522,32 +2522,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
@@ -2564,138 +2564,138 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -2707,32 +2707,32 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -2744,32 +2744,32 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
@@ -2786,27 +2786,27 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
@@ -2823,34 +2823,34 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2860,71 +2860,71 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2934,34 +2934,34 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2971,34 +2971,34 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3008,34 +3008,34 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3045,34 +3045,34 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3082,34 +3082,34 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3119,34 +3119,34 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3156,34 +3156,34 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3193,27 +3193,27 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -3230,27 +3230,27 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -3267,17 +3267,17 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -3287,7 +3287,7 @@
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -3304,27 +3304,27 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -3341,27 +3341,27 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -3378,27 +3378,27 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -3415,27 +3415,27 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -3452,27 +3452,27 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -3489,27 +3489,27 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -3521,32 +3521,32 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -3563,27 +3563,27 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -3600,34 +3600,34 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3637,106 +3637,217 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr">
+      <c r="E92" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F89" t="inlineStr">
+      <c r="F92" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G89" t="inlineStr">
+      <c r="G92" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G89"/>
+  <autoFilter ref="A1:G92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-26
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$92</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$93</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G92"/>
+  <dimension ref="A1:G93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,37 +482,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Firstlead GmbH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ireland,  Spain,  UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Presales Engineer (German Speaking)</t>
+          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Angular, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
+          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
         </is>
       </c>
     </row>
@@ -534,22 +534,22 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ireland,  UK</t>
+          <t>Ireland,  Spain,  UK</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Presales Engineer</t>
+          <t>Presales Engineer (German Speaking)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
+          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
         </is>
       </c>
     </row>
@@ -561,39 +561,39 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Malt</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Ireland,  UK</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Engineering Manager - Payment</t>
+          <t>Presales Engineer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
+          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,27 +603,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Malt</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
+          <t>Senior Engineering Manager - Payment</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
         </is>
       </c>
     </row>
@@ -650,7 +650,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
+          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -660,7 +660,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
         </is>
       </c>
     </row>
@@ -672,32 +672,32 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
+          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Software Engineering Director</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
+          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
         </is>
       </c>
     </row>
@@ -751,64 +751,64 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Banyan Software</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Belgium,  Germany,  Netherlands,  UK</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Software Engineering Director</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
+          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Banyan Software</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Breda, Noord-Brabant, Nederland</t>
+          <t>Belgium,  Germany,  Netherlands,  UK</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
+          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Zoetermeer, Zuid-Holland, Nederland</t>
+          <t>Breda, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -845,7 +845,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
         </is>
       </c>
     </row>
@@ -862,27 +862,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
+          <t>Zoetermeer, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Staff Engineer - Fullstack - Actions</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
         </is>
       </c>
     </row>
@@ -904,22 +904,22 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Join Our Talent Community: Solutions Engineer</t>
+          <t>Staff Engineer - Fullstack - Actions</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
         </is>
       </c>
     </row>
@@ -931,22 +931,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>EMEA</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Engineering Director - Commercial Systems</t>
+          <t>Join Our Talent Community: Solutions Engineer</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -956,7 +956,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
         </is>
       </c>
     </row>
@@ -968,32 +968,32 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Banyansoftware</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>EMEA</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Engineering Director - Commercial Systems</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
+          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
         </is>
       </c>
     </row>
@@ -1010,27 +1010,27 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Banyansoftware</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Staff Software Engineer, Payments</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Payments Platform</t>
+          <t>Staff Software Engineer, Payments</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1067,44 +1067,44 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>AI Software Engineer</t>
+          <t>Senior Software Engineer, Payments Platform</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
         </is>
       </c>
     </row>
@@ -1116,32 +1116,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
+          <t>AI Software Engineer</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
+          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
         </is>
       </c>
     </row>
@@ -1168,17 +1168,17 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
+          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript</t>
+          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
         </is>
       </c>
     </row>
@@ -1195,27 +1195,27 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Grip</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Principal Engineer (Software Engineering/Devops)</t>
+          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
         </is>
       </c>
     </row>
@@ -1232,34 +1232,34 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GradeMatch</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Eindhoven, Noord-Brabant, Nederland</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Full Stack Developer</t>
+          <t>Principal Engineer (Software Engineering/Devops)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1269,34 +1269,34 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Coreweave</t>
+          <t>GradeMatch</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Eindhoven, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Account Solution Architect</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1306,27 +1306,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
@@ -1338,32 +1338,32 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
@@ -1375,32 +1375,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
@@ -1417,64 +1417,64 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
@@ -1486,32 +1486,32 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
@@ -1523,69 +1523,69 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -1612,17 +1612,17 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -1639,27 +1639,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -1676,27 +1676,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -1713,27 +1713,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
@@ -1750,17 +1750,17 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -1770,7 +1770,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
@@ -1787,27 +1787,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
@@ -1834,7 +1834,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
@@ -1856,76 +1856,76 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1935,27 +1935,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
@@ -1972,34 +1972,34 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2009,27 +2009,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -2046,27 +2046,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
@@ -2093,17 +2093,17 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
@@ -2120,27 +2120,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
@@ -2157,27 +2157,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
@@ -2194,34 +2194,34 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2231,27 +2231,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -2268,27 +2268,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -2300,32 +2300,32 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
@@ -2337,32 +2337,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
@@ -2389,17 +2389,17 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
@@ -2416,27 +2416,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
@@ -2458,29 +2458,29 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2490,27 +2490,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -2522,32 +2522,32 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
@@ -2559,32 +2559,32 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
@@ -2611,17 +2611,17 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
@@ -2638,17 +2638,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -2658,7 +2658,7 @@
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
@@ -2675,64 +2675,64 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -2749,27 +2749,27 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -2786,27 +2786,27 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
@@ -2818,32 +2818,32 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -2880,7 +2880,7 @@
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
@@ -2892,32 +2892,32 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
@@ -2929,39 +2929,39 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2971,27 +2971,27 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
@@ -3008,34 +3008,34 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3045,27 +3045,27 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
@@ -3082,27 +3082,27 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
@@ -3119,34 +3119,34 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3156,27 +3156,27 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
@@ -3193,34 +3193,34 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3230,27 +3230,27 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -3277,17 +3277,17 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -3304,27 +3304,27 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -3341,7 +3341,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3351,17 +3351,17 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -3388,17 +3388,17 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -3415,27 +3415,27 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -3452,7 +3452,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3462,17 +3462,17 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -3489,27 +3489,27 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -3526,27 +3526,27 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -3573,17 +3573,17 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3610,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -3632,32 +3632,32 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
@@ -3711,64 +3711,64 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>autoscout24</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
         </is>
       </c>
     </row>
@@ -3785,27 +3785,27 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Sporty Group</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Frontend Engineering Team Lead - MarTech</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
         </is>
       </c>
     </row>
@@ -3817,37 +3817,74 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E92" t="inlineStr">
+      <c r="E93" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F92" t="inlineStr">
+      <c r="F93" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G92" t="inlineStr">
+      <c r="G93" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G92"/>
+  <autoFilter ref="A1:G93"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-27
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$93</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$94</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G93"/>
+  <dimension ref="A1:G94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,74 +482,74 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Firstlead GmbH</t>
+          <t>Ping Identity</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
+          <t>Technical Account Manager</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Angular, Docker, Kubernetes</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
+          <t>https://jobicy.com/jobs/157348-technical-account-manager-10</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Firstlead GmbH</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Ireland,  Spain,  UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Presales Engineer (German Speaking)</t>
+          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Angular, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
+          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
         </is>
       </c>
     </row>
@@ -571,22 +571,22 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ireland,  UK</t>
+          <t>Ireland,  Spain,  UK</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Presales Engineer</t>
+          <t>Presales Engineer (German Speaking)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
+          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
         </is>
       </c>
     </row>
@@ -598,39 +598,39 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Malt</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Ireland,  UK</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Senior Engineering Manager - Payment</t>
+          <t>Presales Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
+          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,27 +640,27 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Malt</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
+          <t>Senior Engineering Manager - Payment</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
         </is>
       </c>
     </row>
@@ -687,7 +687,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
+          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
         </is>
       </c>
     </row>
@@ -709,32 +709,32 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
+          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
         </is>
       </c>
     </row>
@@ -761,7 +761,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Software Engineering Director</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -771,7 +771,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
+          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
         </is>
       </c>
     </row>
@@ -788,64 +788,64 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Banyan Software</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Belgium,  Germany,  Netherlands,  UK</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Software Engineering Director</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
+          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Banyan Software</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Breda, Noord-Brabant, Nederland</t>
+          <t>Belgium,  Germany,  Netherlands,  UK</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
+          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
         </is>
       </c>
     </row>
@@ -867,12 +867,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Zoetermeer, Zuid-Holland, Nederland</t>
+          <t>Breda, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -882,7 +882,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
         </is>
       </c>
     </row>
@@ -899,27 +899,27 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
+          <t>Zoetermeer, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Staff Engineer - Fullstack - Actions</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
         </is>
       </c>
     </row>
@@ -941,22 +941,22 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Join Our Talent Community: Solutions Engineer</t>
+          <t>Staff Engineer - Fullstack - Actions</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
         </is>
       </c>
     </row>
@@ -968,22 +968,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EMEA</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Engineering Director - Commercial Systems</t>
+          <t>Join Our Talent Community: Solutions Engineer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -993,7 +993,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
         </is>
       </c>
     </row>
@@ -1005,32 +1005,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Banyansoftware</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>EMEA</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Engineering Director - Commercial Systems</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
+          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
         </is>
       </c>
     </row>
@@ -1047,27 +1047,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Banyansoftware</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Staff Software Engineer, Payments</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Payments Platform</t>
+          <t>Staff Software Engineer, Payments</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1104,44 +1104,44 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>AI Software Engineer</t>
+          <t>Senior Software Engineer, Payments Platform</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
         </is>
       </c>
     </row>
@@ -1153,32 +1153,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
+          <t>AI Software Engineer</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
+          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
         </is>
       </c>
     </row>
@@ -1205,17 +1205,17 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
+          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript</t>
+          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
         </is>
       </c>
     </row>
@@ -1232,27 +1232,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Grip</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Principal Engineer (Software Engineering/Devops)</t>
+          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
         </is>
       </c>
     </row>
@@ -1269,34 +1269,34 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GradeMatch</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Eindhoven, Noord-Brabant, Nederland</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Full Stack Developer</t>
+          <t>Principal Engineer (Software Engineering/Devops)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1306,34 +1306,34 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Coreweave</t>
+          <t>GradeMatch</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Eindhoven, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Account Solution Architect</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1343,27 +1343,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
@@ -1375,32 +1375,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
@@ -1412,32 +1412,32 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
@@ -1454,64 +1454,64 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
@@ -1523,32 +1523,32 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
@@ -1560,69 +1560,69 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -1649,17 +1649,17 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -1676,27 +1676,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -1713,27 +1713,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -1750,27 +1750,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
@@ -1787,17 +1787,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
@@ -1824,27 +1824,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
@@ -1871,7 +1871,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -1881,7 +1881,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
@@ -1893,76 +1893,76 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1972,27 +1972,27 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
@@ -2009,34 +2009,34 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2046,27 +2046,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -2083,27 +2083,27 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
@@ -2130,17 +2130,17 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
@@ -2157,27 +2157,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
@@ -2194,27 +2194,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
@@ -2231,34 +2231,34 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2268,27 +2268,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -2305,27 +2305,27 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -2337,32 +2337,32 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
@@ -2374,32 +2374,32 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
@@ -2426,17 +2426,17 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
@@ -2453,27 +2453,27 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
@@ -2495,29 +2495,29 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2527,27 +2527,27 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -2559,32 +2559,32 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
@@ -2596,32 +2596,32 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
@@ -2648,17 +2648,17 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
@@ -2675,17 +2675,17 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -2695,7 +2695,7 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
@@ -2712,64 +2712,64 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -2786,27 +2786,27 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -2823,27 +2823,27 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
@@ -2855,32 +2855,32 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
@@ -2907,7 +2907,7 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -2917,7 +2917,7 @@
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
@@ -2929,32 +2929,32 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
@@ -2966,39 +2966,39 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3008,27 +3008,27 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
@@ -3045,34 +3045,34 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3082,27 +3082,27 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
@@ -3119,27 +3119,27 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
@@ -3156,34 +3156,34 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3193,27 +3193,27 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
@@ -3230,34 +3230,34 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3267,27 +3267,27 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -3314,17 +3314,17 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -3341,27 +3341,27 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3388,17 +3388,17 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -3425,17 +3425,17 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -3452,27 +3452,27 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -3499,17 +3499,17 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -3526,27 +3526,27 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -3563,27 +3563,27 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -3610,17 +3610,17 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3647,7 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
@@ -3657,7 +3657,7 @@
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -3669,32 +3669,32 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
@@ -3748,64 +3748,64 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>autoscout24</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
         </is>
       </c>
     </row>
@@ -3822,27 +3822,27 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Sporty Group</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Frontend Engineering Team Lead - MarTech</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
         </is>
       </c>
     </row>
@@ -3854,37 +3854,74 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D94" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr">
+      <c r="E94" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F93" t="inlineStr">
+      <c r="F94" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G93" t="inlineStr">
+      <c r="G94" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G93"/>
+  <autoFilter ref="A1:G94"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-28
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$94</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$98</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G98"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,175 +482,175 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Ping Identity</t>
+          <t>Superchat</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Berlin, Berlin</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Technical Account Manager</t>
+          <t>Tech Lead (m/f/d)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157348-technical-account-manager-10</t>
+          <t>https://www.arbeitnow.com/jobs/companies/superchat/tech-lead-berlin-berlin-146815</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Firstlead GmbH</t>
+          <t>Maze</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Canada,  Ireland,  Netherlands,  Portugal,  Spain,  UK</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
+          <t>Senior Full Stack Product Engineer (TypeScript)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Angular, Docker, Kubernetes</t>
+          <t>React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
+          <t>https://jobicy.com/jobs/151824-senior-full-stack-product-engineer-typescript</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ireland,  Spain,  UK</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Presales Engineer (German Speaking)</t>
+          <t>Senior Forward Deployed Engineer (Technical Data Architect)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>TypeScript, AWS</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/senior-forward-deployed-engineer-technical-data-architect-london-464919</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ireland,  UK</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Presales Engineer</t>
+          <t>Senior Software Engineer - Fullstack</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/databricks/senior-software-engineer-fullstack-amsterdam-449365</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Malt</t>
+          <t>Ping Identity</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Senior Engineering Manager - Payment</t>
+          <t>Technical Account Manager</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -660,14 +660,14 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
+          <t>https://jobicy.com/jobs/157348-technical-account-manager-10</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -677,71 +677,71 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Firstlead GmbH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
+          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Angular, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
+          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Ireland,  Spain,  UK</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
+          <t>Presales Engineer (German Speaking)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
+          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -751,64 +751,64 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Ireland,  UK</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
+          <t>Presales Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
+          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Malt</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Software Engineering Director</t>
+          <t>Senior Engineering Manager - Payment</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
         </is>
       </c>
     </row>
@@ -820,39 +820,39 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Banyan Software</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Belgium,  Germany,  Netherlands,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -862,138 +862,138 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Breda, Noord-Brabant, Nederland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
+          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Zoetermeer, Zuid-Holland, Nederland</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
+          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Staff Engineer - Fullstack - Actions</t>
+          <t>Software Engineering Director</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
+          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Banyan Software</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
+          <t>Belgium,  Germany,  Netherlands,  UK</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Join Our Talent Community: Solutions Engineer</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
+          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
         </is>
       </c>
     </row>
@@ -1005,32 +1005,32 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EMEA</t>
+          <t>Breda, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Engineering Director - Commercial Systems</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
         </is>
       </c>
     </row>
@@ -1047,27 +1047,27 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Banyansoftware</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Zoetermeer, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
         </is>
       </c>
     </row>
@@ -1084,27 +1084,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Staff Software Engineer, Payments</t>
+          <t>Staff Engineer - Fullstack - Actions</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
         </is>
       </c>
     </row>
@@ -1121,34 +1121,34 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Payments Platform</t>
+          <t>Join Our Talent Community: Solutions Engineer</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1158,34 +1158,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>EMEA</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>AI Software Engineer</t>
+          <t>Engineering Director - Commercial Systems</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
+          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,34 +1195,34 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Banyansoftware</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1232,34 +1232,34 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
+          <t>Staff Software Engineer, Payments</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1269,27 +1269,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Grip</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Principal Engineer (Software Engineering/Devops)</t>
+          <t>Senior Software Engineer, Payments Platform</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
         </is>
       </c>
     </row>
@@ -1301,39 +1301,39 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>GradeMatch</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Eindhoven, Noord-Brabant, Nederland</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Full Stack Developer</t>
+          <t>AI Software Engineer</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
+          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1343,34 +1343,34 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Coreweave</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Account Solution Architect</t>
+          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1380,54 +1380,54 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Principal Engineer (Software Engineering/Devops)</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -1437,14 +1437,14 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1454,34 +1454,34 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>GradeMatch</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Eindhoven, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>Java, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1491,145 +1491,145 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1639,71 +1639,71 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1713,64 +1713,64 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -1787,27 +1787,27 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -1824,27 +1824,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -1861,27 +1861,27 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -1898,27 +1898,27 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
@@ -1930,39 +1930,39 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1972,34 +1972,34 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2009,34 +2009,34 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2046,71 +2046,71 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2120,34 +2120,34 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2157,34 +2157,34 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2194,27 +2194,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -2231,27 +2231,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
@@ -2268,34 +2268,34 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -2305,34 +2305,34 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2342,71 +2342,71 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2416,27 +2416,27 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -2453,27 +2453,27 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -2490,27 +2490,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
@@ -2522,39 +2522,39 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2564,12 +2564,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -2584,51 +2584,51 @@
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2638,34 +2638,34 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2675,27 +2675,27 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -2712,27 +2712,27 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
@@ -2744,150 +2744,150 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2897,27 +2897,27 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -2929,32 +2929,32 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -2971,27 +2971,27 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
@@ -3003,39 +3003,39 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3045,34 +3045,34 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3082,71 +3082,71 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3156,34 +3156,34 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -3193,34 +3193,34 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3230,34 +3230,34 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3267,7 +3267,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3277,24 +3277,24 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3304,34 +3304,34 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3341,34 +3341,34 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3378,34 +3378,34 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3415,27 +3415,27 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -3452,27 +3452,27 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -3489,27 +3489,27 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -3526,27 +3526,27 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -3563,27 +3563,27 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -3600,27 +3600,27 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -3637,27 +3637,27 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -3674,27 +3674,27 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -3706,32 +3706,32 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -3748,27 +3748,27 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -3785,71 +3785,71 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3859,69 +3859,217 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D98" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr">
+      <c r="E98" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F94" t="inlineStr">
+      <c r="F98" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G94" t="inlineStr">
+      <c r="G98" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G94"/>
+  <autoFilter ref="A1:G98"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-29
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$98</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$104</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G98"/>
+  <dimension ref="A1:G104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,155 +482,155 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Superchat</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Berlin, Berlin</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Tech Lead (m/f/d)</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/superchat/tech-lead-berlin-berlin-146815</t>
+          <t>https://jobicy.com/jobs/157787-senior-software-engineer-18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Maze</t>
+          <t>Priva</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Canada,  Ireland,  Netherlands,  Portugal,  Spain,  UK</t>
+          <t>De Lier, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Senior Full Stack Product Engineer (TypeScript)</t>
+          <t>Staff Frontend Engineer</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>React, TypeScript, Kubernetes, AWS</t>
+          <t>Angular, TypeScript</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/151824-senior-full-stack-product-engineer-typescript</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/priva/staff-frontend-engineer-de-lier-72329</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Forward Deployed Engineer (Technical Data Architect)</t>
+          <t>Senior/Staff Application Security Engineer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>TypeScript, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/senior-forward-deployed-engineer-technical-data-architect-london-464919</t>
+          <t>https://jobicy.com/jobs/157528-senior-staff-application-security-engineer</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Europe,  Israel</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Fullstack</t>
+          <t>Senior Site Reliability Engineer (DevTools)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/databricks/senior-software-engineer-fullstack-amsterdam-449365</t>
+          <t>https://jobicy.com/jobs/157510-senior-site-reliability-engineer-devtools</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -640,34 +640,34 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Ping Identity</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Technical Account Manager</t>
+          <t>Senior Product Designer - Compute, Nebius Console</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157348-technical-account-manager-10</t>
+          <t>https://jobicy.com/jobs/157502-senior-product-designer-compute-nebius-console</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -677,7 +677,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Firstlead GmbH</t>
+          <t>easybill GmbH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -687,61 +687,61 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
+          <t>Senior Software Engineer (PHP, TypeScript, Node.js) m/w/d</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Angular, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
+          <t>https://www.arbeitnow.com/jobs/companies/easybill-gmbh/senior-software-engineer-php-typescript-nodejs-berlin-53164</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Superchat</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Ireland,  Spain,  UK</t>
+          <t>Berlin, Berlin</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Presales Engineer (German Speaking)</t>
+          <t>Tech Lead (m/f/d)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
+          <t>https://www.arbeitnow.com/jobs/companies/superchat/tech-lead-berlin-berlin-146815</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -751,34 +751,34 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Maze</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Ireland,  UK</t>
+          <t>Canada,  Ireland,  Netherlands,  Portugal,  Spain,  UK</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Presales Engineer</t>
+          <t>Senior Full Stack Product Engineer (TypeScript)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
+          <t>https://jobicy.com/jobs/151824-senior-full-stack-product-engineer-typescript</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -788,34 +788,34 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Malt</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior Engineering Manager - Payment</t>
+          <t>Senior Forward Deployed Engineer (Technical Data Architect)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>TypeScript, AWS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/senior-forward-deployed-engineer-technical-data-architect-london-464919</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -825,108 +825,108 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
+          <t>Senior Software Engineer - Fullstack</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/databricks/senior-software-engineer-fullstack-amsterdam-449365</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Ping Identity</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
+          <t>Technical Account Manager</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
+          <t>https://jobicy.com/jobs/157348-technical-account-manager-10</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Firstlead GmbH</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
+          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Angular, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
+          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -936,34 +936,34 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Ireland,  Spain,  UK</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Software Engineering Director</t>
+          <t>Presales Engineer (German Speaking)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
+          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -973,34 +973,34 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Banyan Software</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Belgium,  Germany,  Netherlands,  UK</t>
+          <t>Ireland,  UK</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Presales Engineer</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
+          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1010,34 +1010,34 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Malt</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Breda, Noord-Brabant, Nederland</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
+          <t>Senior Engineering Manager - Payment</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1047,34 +1047,34 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Zoetermeer, Zuid-Holland, Nederland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
+          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,71 +1084,71 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Staff Engineer - Fullstack - Actions</t>
+          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Join Our Talent Community: Solutions Engineer</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
+          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1163,44 +1163,44 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>EMEA</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Engineering Director - Commercial Systems</t>
+          <t>Software Engineering Director</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
+          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Banyansoftware</t>
+          <t>Banyan Software</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Belgium,  Germany,  Netherlands,  UK</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -1215,7 +1215,7 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
+          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
         </is>
       </c>
     </row>
@@ -1232,27 +1232,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>Breda, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Staff Software Engineer, Payments</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
         </is>
       </c>
     </row>
@@ -1269,71 +1269,71 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>Zoetermeer, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Payments Platform</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>AI Software Engineer</t>
+          <t>Staff Engineer - Fullstack - Actions</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1343,71 +1343,71 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
+          <t>Join Our Talent Community: Solutions Engineer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EMEA</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
+          <t>Engineering Director - Commercial Systems</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
+          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1417,34 +1417,34 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Grip</t>
+          <t>Banyansoftware</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Principal Engineer (Software Engineering/Devops)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1454,34 +1454,34 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>GradeMatch</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Eindhoven, Noord-Brabant, Nederland</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Full Stack Developer</t>
+          <t>Staff Software Engineer, Payments</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1491,108 +1491,108 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Coreweave</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Account Solution Architect</t>
+          <t>Senior Software Engineer, Payments Platform</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>AI Software Engineer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1602,34 +1602,34 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1639,71 +1639,71 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Principal Engineer (Software Engineering/Devops)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>GradeMatch</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Eindhoven, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1713,108 +1713,108 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1824,34 +1824,34 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1861,71 +1861,71 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1935,64 +1935,64 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -2009,27 +2009,27 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -2046,27 +2046,27 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -2078,39 +2078,39 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2120,34 +2120,34 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2157,34 +2157,34 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2194,34 +2194,34 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2231,34 +2231,34 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2268,71 +2268,71 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2342,34 +2342,34 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -2379,34 +2379,34 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2416,34 +2416,34 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2453,34 +2453,34 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2490,71 +2490,71 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2564,34 +2564,34 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2601,34 +2601,34 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2638,27 +2638,27 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -2675,34 +2675,34 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2712,34 +2712,34 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2749,34 +2749,34 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2786,34 +2786,34 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2823,34 +2823,34 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2860,34 +2860,34 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2897,71 +2897,71 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2981,61 +2981,61 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -3045,17 +3045,17 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -3065,14 +3065,14 @@
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3082,17 +3082,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -3102,44 +3102,44 @@
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -3151,113 +3151,113 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -3267,34 +3267,34 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -3304,71 +3304,71 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3378,34 +3378,34 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -3415,34 +3415,34 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3452,34 +3452,34 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3489,34 +3489,34 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3526,34 +3526,34 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3563,34 +3563,34 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3600,34 +3600,34 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3637,27 +3637,27 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -3674,27 +3674,27 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -3711,27 +3711,27 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -3748,27 +3748,27 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -3785,27 +3785,27 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -3822,27 +3822,27 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -3854,32 +3854,32 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -3896,27 +3896,27 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -3933,143 +3933,365 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Doctolib</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>Paris, Paris</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Design System Director (x/f/m)</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C98" t="inlineStr">
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D104" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E98" t="inlineStr">
+      <c r="E104" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F98" t="inlineStr">
+      <c r="F104" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G98" t="inlineStr">
+      <c r="G104" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G98"/>
+  <autoFilter ref="A1:G104"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-30
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$104</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$106</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:G106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,44 +482,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Tebi</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Senior Backend Engineer</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes, AWS</t>
+          <t>Java, Kafka, Docker</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157787-senior-software-engineer-18</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tebi/senior-backend-engineer-amsterdam-465520</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,27 +529,27 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Priva</t>
+          <t>Gridty</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>De Lier, Zuid-Holland, Netherlands</t>
+          <t>Cologne</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer</t>
+          <t>Lead Software Engineer / Energie-Startup (m/w/d)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Angular, TypeScript</t>
+          <t>React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/priva/staff-frontend-engineer-de-lier-72329</t>
+          <t>https://www.arbeitnow.com/jobs/companies/gridty/lead-software-engineer-energie-startup-cologne-32422</t>
         </is>
       </c>
     </row>
@@ -566,27 +566,27 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior/Staff Application Security Engineer</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157528-senior-staff-application-security-engineer</t>
+          <t>https://jobicy.com/jobs/157787-senior-software-engineer-18</t>
         </is>
       </c>
     </row>
@@ -598,32 +598,32 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Priva</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Europe,  Israel</t>
+          <t>De Lier, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Senior Site Reliability Engineer (DevTools)</t>
+          <t>Staff Frontend Engineer</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Angular, TypeScript</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157510-senior-site-reliability-engineer-devtools</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/priva/staff-frontend-engineer-de-lier-72329</t>
         </is>
       </c>
     </row>
@@ -650,17 +650,17 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Senior Product Designer - Compute, Nebius Console</t>
+          <t>Senior/Staff Application Security Engineer</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157502-senior-product-designer-compute-nebius-console</t>
+          <t>https://jobicy.com/jobs/157528-senior-staff-application-security-engineer</t>
         </is>
       </c>
     </row>
@@ -672,106 +672,106 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>easybill GmbH</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Europe,  Israel</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (PHP, TypeScript, Node.js) m/w/d</t>
+          <t>Senior Site Reliability Engineer (DevTools)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/easybill-gmbh/senior-software-engineer-php-typescript-nodejs-berlin-53164</t>
+          <t>https://jobicy.com/jobs/157510-senior-site-reliability-engineer-devtools</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Superchat</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Berlin, Berlin</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Tech Lead (m/f/d)</t>
+          <t>Senior Product Designer - Compute, Nebius Console</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/superchat/tech-lead-berlin-berlin-146815</t>
+          <t>https://jobicy.com/jobs/157502-senior-product-designer-compute-nebius-console</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Maze</t>
+          <t>easybill GmbH</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Canada,  Ireland,  Netherlands,  Portugal,  Spain,  UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Full Stack Product Engineer (TypeScript)</t>
+          <t>Senior Software Engineer (PHP, TypeScript, Node.js) m/w/d</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/151824-senior-full-stack-product-engineer-typescript</t>
+          <t>https://www.arbeitnow.com/jobs/companies/easybill-gmbh/senior-software-engineer-php-typescript-nodejs-berlin-53164</t>
         </is>
       </c>
     </row>
@@ -788,27 +788,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Superchat</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Berlin, Berlin</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Senior Forward Deployed Engineer (Technical Data Architect)</t>
+          <t>Tech Lead (m/f/d)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>TypeScript, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/senior-forward-deployed-engineer-technical-data-architect-london-464919</t>
+          <t>https://www.arbeitnow.com/jobs/companies/superchat/tech-lead-berlin-berlin-146815</t>
         </is>
       </c>
     </row>
@@ -820,76 +820,76 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Maze</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Canada,  Ireland,  Netherlands,  Portugal,  Spain,  UK</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Fullstack</t>
+          <t>Senior Full Stack Product Engineer (TypeScript)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/databricks/senior-software-engineer-fullstack-amsterdam-449365</t>
+          <t>https://jobicy.com/jobs/151824-senior-full-stack-product-engineer-typescript</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Ping Identity</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Technical Account Manager</t>
+          <t>Senior Forward Deployed Engineer (Technical Data Architect)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>TypeScript, AWS</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157348-technical-account-manager-10</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/senior-forward-deployed-engineer-technical-data-architect-london-464919</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -899,34 +899,34 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Firstlead GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
+          <t>Senior Software Engineer - Fullstack</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Angular, Docker, Kubernetes</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/databricks/senior-software-engineer-fullstack-amsterdam-449365</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -936,64 +936,64 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Ping Identity</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Ireland,  Spain,  UK</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Presales Engineer (German Speaking)</t>
+          <t>Technical Account Manager</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
+          <t>https://jobicy.com/jobs/157348-technical-account-manager-10</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Firstlead GmbH</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Ireland,  UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Presales Engineer</t>
+          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Angular, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
+          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
         </is>
       </c>
     </row>
@@ -1005,76 +1005,76 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Malt</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Ireland,  Spain,  UK</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Senior Engineering Manager - Payment</t>
+          <t>Presales Engineer (German Speaking)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
+          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Ireland,  UK</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
+          <t>Presales Engineer</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
+          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,27 +1084,27 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Malt</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
+          <t>Senior Engineering Manager - Payment</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
         </is>
       </c>
     </row>
@@ -1116,32 +1116,32 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
+          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
         </is>
       </c>
     </row>
@@ -1153,32 +1153,32 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Software Engineering Director</t>
+          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
         </is>
       </c>
     </row>
@@ -1195,101 +1195,101 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Banyan Software</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Belgium,  Germany,  Netherlands,  UK</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
+          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Breda, Noord-Brabant, Nederland</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
+          <t>Software Engineering Director</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
+          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Banyan Software</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Zoetermeer, Zuid-Holland, Nederland</t>
+          <t>Belgium,  Germany,  Netherlands,  UK</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
+          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
         </is>
       </c>
     </row>
@@ -1306,27 +1306,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
+          <t>Breda, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Staff Engineer - Fullstack - Actions</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
         </is>
       </c>
     </row>
@@ -1343,27 +1343,27 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
+          <t>Zoetermeer, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Join Our Talent Community: Solutions Engineer</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
         </is>
       </c>
     </row>
@@ -1375,32 +1375,32 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>EMEA</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Engineering Director - Commercial Systems</t>
+          <t>Staff Engineer - Fullstack - Actions</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
         </is>
       </c>
     </row>
@@ -1417,27 +1417,27 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Banyansoftware</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Join Our Talent Community: Solutions Engineer</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
         </is>
       </c>
     </row>
@@ -1449,32 +1449,32 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>EMEA</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Staff Software Engineer, Payments</t>
+          <t>Engineering Director - Commercial Systems</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
+          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
         </is>
       </c>
     </row>
@@ -1491,71 +1491,71 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Banyansoftware</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Payments Platform</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>AI Software Engineer</t>
+          <t>Staff Software Engineer, Payments</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1565,27 +1565,27 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
+          <t>Senior Software Engineer, Payments Platform</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
         </is>
       </c>
     </row>
@@ -1597,32 +1597,32 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
+          <t>AI Software Engineer</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
+          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
         </is>
       </c>
     </row>
@@ -1639,27 +1639,27 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Grip</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Principal Engineer (Software Engineering/Devops)</t>
+          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
         </is>
       </c>
     </row>
@@ -1676,34 +1676,34 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>GradeMatch</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Eindhoven, Noord-Brabant, Nederland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Full Stack Developer</t>
+          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1713,34 +1713,34 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Coreweave</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Account Solution Architect</t>
+          <t>Principal Engineer (Software Engineering/Devops)</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1750,64 +1750,64 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>GradeMatch</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>Eindhoven, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>Java, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
@@ -1824,27 +1824,27 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
@@ -1856,76 +1856,76 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1935,27 +1935,27 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1982,24 +1982,24 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2009,64 +2009,64 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -2083,27 +2083,27 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -2120,27 +2120,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -2157,27 +2157,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -2194,27 +2194,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
@@ -2231,27 +2231,27 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
@@ -2268,27 +2268,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
@@ -2300,39 +2300,39 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -2342,71 +2342,71 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2416,34 +2416,34 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2453,34 +2453,34 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2490,27 +2490,27 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -2527,27 +2527,27 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
@@ -2564,27 +2564,27 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
@@ -2601,27 +2601,27 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
@@ -2638,34 +2638,34 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2675,34 +2675,34 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2712,27 +2712,27 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -2744,32 +2744,32 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -2786,27 +2786,27 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
@@ -2818,32 +2818,32 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
@@ -2860,27 +2860,27 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
@@ -2897,34 +2897,34 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2934,64 +2934,64 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -3008,27 +3008,27 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
@@ -3040,32 +3040,32 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
@@ -3082,27 +3082,27 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
@@ -3119,101 +3119,101 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -3230,27 +3230,27 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -3262,32 +3262,32 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
@@ -3299,32 +3299,32 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
@@ -3336,32 +3336,32 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
@@ -3378,71 +3378,71 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -3452,34 +3452,34 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -3489,34 +3489,34 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3526,27 +3526,27 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
@@ -3563,34 +3563,34 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -3600,34 +3600,34 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3637,34 +3637,34 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -3674,34 +3674,34 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3711,27 +3711,27 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -3748,27 +3748,27 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -3785,27 +3785,27 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -3822,7 +3822,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3832,17 +3832,17 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -3859,27 +3859,27 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -3896,27 +3896,27 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -3933,27 +3933,27 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -3970,27 +3970,27 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -4007,27 +4007,27 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -4054,17 +4054,17 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
@@ -4076,32 +4076,32 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
@@ -4118,27 +4118,27 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
@@ -4150,106 +4150,106 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Dataiku</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Fullstack Software Engineer - Core</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Baringa</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Senior Software Engineer - Future Opportunities</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>autoscout24</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
         </is>
       </c>
     </row>
@@ -4261,37 +4261,111 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr">
+      <c r="D106" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E104" t="inlineStr">
+      <c r="E106" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F104" t="inlineStr">
+      <c r="F106" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G104" t="inlineStr">
+      <c r="G106" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G104"/>
+  <autoFilter ref="A1:G106"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Job tracker update 2026-10-31
</commit_message>
<xml_diff>
--- a/data/job_history.xlsx
+++ b/data/job_history.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Job History (30 days)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$106</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Job History (30 days)'!$A$1:$G$111</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -430,7 +430,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G106"/>
+  <dimension ref="A1:G111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -492,34 +492,34 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Tebi</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Senior Backend Engineer</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Java, Kafka, Docker</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tebi/senior-backend-engineer-amsterdam-465520</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-371554</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-10-30</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -529,34 +529,34 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Gridty</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Cologne</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lead Software Engineer / Energie-Startup (m/w/d)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/gridty/lead-software-engineer-energie-startup-cologne-32422</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-295419</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -566,34 +566,34 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>ecosio</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Ireland</t>
+          <t>Austria,  Croatia,  Germany,  Hungary,  Italy,  Portugal,  Spain,  UK</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Senior Software Engineer</t>
+          <t>Full Stack Developer - Java &amp; React (f/m/d)</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157787-senior-software-engineer-18</t>
+          <t>https://jobicy.com/jobs/158154-full-stack-developer-java-react-f-m-d-2</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -603,138 +603,138 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Priva</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>De Lier, Zuid-Holland, Netherlands</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer</t>
+          <t>Senior Fullstack Engineer - Java, React (x/f/m)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Angular, TypeScript</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/priva/staff-frontend-engineer-de-lier-72329</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/doctolib/senior-fullstack-engineer-java-react-amsterdam-35344</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-31</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Deliveroo</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Senior/Staff Application Security Engineer</t>
+          <t>Senior Software Engineer (Fullstack) - Merchant EMEA</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157528-senior-staff-application-security-engineer</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/deliveroo/senior-software-engineer-fullstack-merchant-emea-london-1521</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Tebi</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Europe,  Israel</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Senior Site Reliability Engineer (DevTools)</t>
+          <t>Senior Backend Engineer</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Kafka, Docker</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157510-senior-site-reliability-engineer-devtools</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tebi/senior-backend-engineer-amsterdam-465520</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-10-29</t>
+          <t>2026-10-30</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Gridty</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Cologne</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Senior Product Designer - Compute, Nebius Console</t>
+          <t>Lead Software Engineer / Energie-Startup (m/w/d)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157502-senior-product-designer-compute-nebius-console</t>
+          <t>https://www.arbeitnow.com/jobs/companies/gridty/lead-software-engineer-energie-startup-cologne-32422</t>
         </is>
       </c>
     </row>
@@ -746,39 +746,39 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>easybill GmbH</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Ireland</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (PHP, TypeScript, Node.js) m/w/d</t>
+          <t>Senior Software Engineer</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/easybill-gmbh/senior-software-engineer-php-typescript-nodejs-berlin-53164</t>
+          <t>https://jobicy.com/jobs/157787-senior-software-engineer-18</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -788,34 +788,34 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Superchat</t>
+          <t>Priva</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Berlin, Berlin</t>
+          <t>De Lier, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Tech Lead (m/f/d)</t>
+          <t>Staff Frontend Engineer</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Angular, TypeScript</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/superchat/tech-lead-berlin-berlin-146815</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/priva/staff-frontend-engineer-de-lier-72329</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -825,145 +825,145 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Maze</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Canada,  Ireland,  Netherlands,  Portugal,  Spain,  UK</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Senior Full Stack Product Engineer (TypeScript)</t>
+          <t>Senior/Staff Application Security Engineer</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>React, TypeScript, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/151824-senior-full-stack-product-engineer-typescript</t>
+          <t>https://jobicy.com/jobs/157528-senior-staff-application-security-engineer</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Europe,  Israel</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Senior Forward Deployed Engineer (Technical Data Architect)</t>
+          <t>Senior Site Reliability Engineer (DevTools)</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>TypeScript, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/senior-forward-deployed-engineer-technical-data-architect-london-464919</t>
+          <t>https://jobicy.com/jobs/157510-senior-site-reliability-engineer-devtools</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-10-28</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Fullstack</t>
+          <t>Senior Product Designer - Compute, Nebius Console</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/databricks/senior-software-engineer-fullstack-amsterdam-449365</t>
+          <t>https://jobicy.com/jobs/157502-senior-product-designer-compute-nebius-console</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-10-27</t>
+          <t>2026-10-29</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Ping Identity</t>
+          <t>easybill GmbH</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Technical Account Manager</t>
+          <t>Senior Software Engineer (PHP, TypeScript, Node.js) m/w/d</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/157348-technical-account-manager-10</t>
+          <t>https://www.arbeitnow.com/jobs/companies/easybill-gmbh/senior-software-engineer-php-typescript-nodejs-berlin-53164</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -973,34 +973,34 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Firstlead GmbH</t>
+          <t>Superchat</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Berlin, Berlin</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
+          <t>Tech Lead (m/f/d)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Angular, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
+          <t>https://www.arbeitnow.com/jobs/companies/superchat/tech-lead-berlin-berlin-146815</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1010,71 +1010,71 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>Maze</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Ireland,  Spain,  UK</t>
+          <t>Canada,  Ireland,  Netherlands,  Portugal,  Spain,  UK</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Presales Engineer (German Speaking)</t>
+          <t>Senior Full Stack Product Engineer (TypeScript)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
+          <t>https://jobicy.com/jobs/151824-senior-full-stack-product-engineer-typescript</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Twilio</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Ireland,  UK</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Presales Engineer</t>
+          <t>Senior Forward Deployed Engineer (Technical Data Architect)</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>TypeScript, AWS</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/senior-forward-deployed-engineer-technical-data-architect-london-464919</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-28</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1084,71 +1084,71 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Malt</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>Senior Engineering Manager - Payment</t>
+          <t>Senior Software Engineer - Fullstack</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/databricks/senior-software-engineer-fullstack-amsterdam-449365</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Ping Identity</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
+          <t>Technical Account Manager</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
+          <t>https://jobicy.com/jobs/157348-technical-account-manager-10</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-26</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1158,34 +1158,34 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Firstlead GmbH</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
+          <t>CTO (m/w/d) – Tech-Lead mit strategischem Weitblick &amp; Hands-on-Mentalität</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Angular, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
+          <t>https://www.arbeitnow.com/jobs/companies/firstlead-gmbh/cto-tech-lead-mit-strategischem-weitblick-hands-on-mentalitat-berlin-231155</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1195,34 +1195,34 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Ireland,  Spain,  UK</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>Engineering Manager</t>
+          <t>Presales Engineer (German Speaking)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
+          <t>https://jobicy.com/jobs/156791-presales-engineer-german-speaking</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1232,71 +1232,71 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Twilio</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Anywhere</t>
+          <t>Ireland,  UK</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Software Engineering Director</t>
+          <t>Presales Engineer</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
+          <t>https://jobicy.com/jobs/156788-presales-engineer</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-10-24</t>
+          <t>2026-10-25</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Banyan Software</t>
+          <t>Malt</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Belgium,  Germany,  Netherlands,  UK</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior Engineering Manager - Payment</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/malt/senior-engineering-manager-payment-paris-261962</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1306,34 +1306,34 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Breda, Noord-Brabant, Nederland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
+          <t>Senior AI Engineer - Search &amp; Recommendation - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-search-recommendation-patient-team-paris-paris-428774</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1343,108 +1343,108 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Whitevision B.V.</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Zoetermeer, Zuid-Holland, Nederland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
+          <t>Senior AI Engineer - Patient Team (x/f/m)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ai-engineer-patient-team-paris-paris-437192</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>Staff Engineer - Fullstack - Actions</t>
+          <t>Engineering Manager</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
+          <t>https://jobicy.com/jobs/149575-engineering-manager</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Staffbase</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
+          <t>Anywhere</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>Join Our Talent Community: Solutions Engineer</t>
+          <t>Software Engineering Director</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
+          <t>https://jobicy.com/jobs/149571-software-engineering-director</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1454,27 +1454,27 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Canonical</t>
+          <t>Banyan Software</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>EMEA</t>
+          <t>Belgium,  Germany,  Netherlands,  UK</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>Engineering Director - Commercial Systems</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
+          <t>https://jobicy.com/jobs/156602-forward-deployed-engineer-8</t>
         </is>
       </c>
     </row>
@@ -1491,27 +1491,27 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Banyansoftware</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Breda, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Breda</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-breda-408432</t>
         </is>
       </c>
     </row>
@@ -1528,27 +1528,27 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Whitevision B.V.</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>Zoetermeer, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Staff Software Engineer, Payments</t>
+          <t>Senior Implementatie Consultant SaaS, €4.250 – €6.000 | Zoetermeer</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/whitevision-bv/senior-implementatie-consultant-saas-eur4250-eur6000-zoetermeer-271006</t>
         </is>
       </c>
     </row>
@@ -1565,108 +1565,108 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Airwallex</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>NL - Amsterdam</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Payments Platform</t>
+          <t>Staff Engineer - Fullstack - Actions</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Docker</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/staff-engineer-fullstack-actions-berlin-chemnitz-sachsen-dresden-sachsen-256251</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Staffbase</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Berlin; Chemnitz, Sachsen; Dresden, Sachsen; Köln, Nordrhein-Westfalen; München, Bayern</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>AI Software Engineer</t>
+          <t>Join Our Talent Community: Solutions Engineer</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
+          <t>https://www.arbeitnow.com/jobs/companies/staffbase/join-our-talent-community-solutions-engineer-berlin-chemnitz-sachsen-dresden-sachsen-koln-nordrhein-westfalen-munchen-bayern-181611</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Canonical</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EMEA</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
+          <t>Engineering Director - Commercial Systems</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
+          <t>https://jobicy.com/jobs/156570-engineering-director-commercial-systems</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1676,34 +1676,34 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>TecFox GmbH</t>
+          <t>Banyansoftware</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/banyansoftware/forward-deployed-engineer-354025</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1713,34 +1713,34 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Grip</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Principal Engineer (Software Engineering/Devops)</t>
+          <t>Staff Software Engineer, Payments</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/staff-software-engineer-payments-amsterdam-298606</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-23</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1750,71 +1750,71 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GradeMatch</t>
+          <t>Airwallex</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Eindhoven, Noord-Brabant, Nederland</t>
+          <t>NL - Amsterdam</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Full Stack Developer</t>
+          <t>Senior Software Engineer, Payments Platform</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript</t>
+          <t>Java, Spring Boot, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/airwallex/senior-software-engineer-payments-platform-amsterdam-175739</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Coreweave</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Account Solution Architect</t>
+          <t>AI Software Engineer</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
+          <t>https://jobicy.com/jobs/153823-ai-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1824,71 +1824,71 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Swisscom</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Netherlands</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Senior DevOps Engineer</t>
+          <t>Senior Fullstack-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular</t>
+          <t>Java, Spring Boot, Angular, React, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-fullstack-softwareentwickler-berlin-133162</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>TecFox GmbH</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Senior Frontend-Softwareentwickler (m/w/d)</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
+          <t>https://www.arbeitnow.com/jobs/companies/tecfox-gmbh/senior-frontend-softwareentwickler-berlin-422309</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1898,34 +1898,34 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Buying Labs</t>
+          <t>Grip</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Engineer (m/f/d)</t>
+          <t>Principal Engineer (Software Engineering/Devops)</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/grip/remote-principal-engineer-software-engineering-devops-62745</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1935,71 +1935,71 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Andercore</t>
+          <t>GradeMatch</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Eindhoven, Noord-Brabant, Nederland</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Staff Engineer</t>
+          <t>Full Stack Developer</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, Angular, React, TypeScript</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/gradematch/full-stack-developer-eindhoven-293496</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Skedda</t>
+          <t>Coreweave</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
+          <t>Account Solution Architect</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Java</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/coreweave/account-solution-architect-london-475102</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2009,34 +2009,34 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Natalie Felsinger Consulting</t>
+          <t>Swisscom</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Frechen</t>
+          <t>Rotterdam, Zuid-Holland, Netherlands</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior DevOps Engineer</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, Spring Boot, Angular</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/swisscom/senior-devops-engineer-rotterdam-135896</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2046,34 +2046,34 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bloomreach</t>
+          <t>infisical</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Brazil,  Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
+          <t>Senior Full Stack Engineer</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
+          <t>https://jobicy.com/jobs/155949-senior-full-stack-engineer-8</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2083,34 +2083,34 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Buying Labs</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
+          <t>Senior Full-Stack Engineer (m/f/d)</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>React</t>
+          <t>React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
+          <t>https://www.arbeitnow.com/jobs/companies/buying-labs/senior-full-stack-engineer-hamburg-306603</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-20</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2120,71 +2120,71 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Tether Operations Limited</t>
+          <t>Andercore</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
+          <t>Staff Engineer</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
+          <t>https://www.arbeitnow.com/jobs/companies/andercore/staff-engineer-berlin-165964</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Payter B.V.</t>
+          <t>Skedda</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Rotterdam, Zuid-Holland, Nederland</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Full Stack Tech Lead</t>
+          <t>Senior Full-Stack Software Engineer (Remote in Europe)</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
+          <t>Java</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
+          <t>https://jobicy.com/jobs/155727-senior-full-stack-software-engineer-remote-in-europe-2</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2194,64 +2194,64 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Natalie Felsinger Consulting</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Frechen</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
+          <t>https://www.arbeitnow.com/jobs/companies/natalie-felsinger-consulting/senior-java-fullstack-developer-frechen-256898</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MILES Mobility GmbH</t>
+          <t>Bloomreach</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Europe</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Staff Software Engineer - Python, Java / Spring or Go</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, React, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
+          <t>https://jobicy.com/jobs/155731-staff-software-engineer-python-java-spring-or-go</t>
         </is>
       </c>
     </row>
@@ -2268,27 +2268,27 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Eye Security</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Berlin - hybrid</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Agents (m/f/x)</t>
+          <t>Mobile Engineer - React Native (100% Remote) - Worldwide</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/mobile-engineer-react-native-100-remote-worldwide-united-kindom-24659</t>
         </is>
       </c>
     </row>
@@ -2305,27 +2305,27 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Tether Operations Limited</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Senior IA Inference Engineer (x/f/m)</t>
+          <t>Fullstack Engineer - AgenticOps (100% Remote)</t>
         </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>TypeScript</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/tether-operations-limited/fullstack-engineer-agenticops-100-remote-united-kindom-441724</t>
         </is>
       </c>
     </row>
@@ -2342,27 +2342,27 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Payter B.V.</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Rotterdam, Zuid-Holland, Nederland</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Senior Agents Platform Engineer (x/f/m)</t>
+          <t>Full Stack Tech Lead</t>
         </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Java, Angular, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/payter-bv/full-stack-tech-lead-rotterdam-21453</t>
         </is>
       </c>
     </row>
@@ -2374,39 +2374,39 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Apollo.io</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Senior Software Engineer, Growth</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-49699</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-10-17</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -2416,34 +2416,34 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Sereact GmbH</t>
+          <t>MILES Mobility GmbH</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Stuttgart Schockenriedstr. 17</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Cybersecurity Intern</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility-gmbh/senior-react-native-engineer-app-owner-d-berlin-295111</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -2453,34 +2453,34 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>mirakllabs</t>
+          <t>Eye Security</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Berlin - hybrid</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Software Engineer, Agents (m/f/x)</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
+          <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-agents-berlin-285258</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -2490,34 +2490,34 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>idnow</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Rennes, Ille-et-Vilaine</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Solution Engineer (f/m/d)</t>
+          <t>Senior IA Inference Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-ia-inference-engineer-paris-paris-99480</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -2527,71 +2527,71 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Pennylane SAS</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>All France (remote)</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer RoR/JS W/M</t>
+          <t>Senior Agents Platform Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-agents-platform-engineer-paris-paris-164639</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Apollo.io</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Software Engineer Intern - Financial Services</t>
+          <t>Senior Software Engineer, Growth</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
+          <t>React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
+          <t>https://jobicy.com/jobs/155618-senior-software-engineer-growth-2</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-17</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -2601,34 +2601,34 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Mirakl - Labs</t>
+          <t>Sereact GmbH</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Paris, France</t>
+          <t>Stuttgart Schockenriedstr. 17</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Software Engineer Apprentice - Connect</t>
+          <t>Cybersecurity Intern</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Docker</t>
+          <t>TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
+          <t>https://www.arbeitnow.com/jobs/companies/sereact-gmbh/cybersecurity-intern-stuttgart-351050</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2638,34 +2638,34 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Conflux</t>
+          <t>mirakllabs</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Utrecht, Utrecht, Nederland</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Senior Java Developer</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Java, AWS</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakllabs/software-engineer-intern-financial-services-paris-223168</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2675,27 +2675,27 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Adikteev</t>
+          <t>idnow</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Remote job</t>
+          <t>Rennes, Ille-et-Vilaine</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Staff Site Reliability Engineer</t>
+          <t>Solution Engineer (f/m/d)</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>AWS</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/idnow/solution-engineer-rennes-ille-et-vilaine-342860</t>
         </is>
       </c>
     </row>
@@ -2712,34 +2712,34 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Accso – Accelerated Solutions GmbH</t>
+          <t>Pennylane SAS</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Darmstadt</t>
+          <t>All France (remote)</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
+          <t>Fullstack Software Engineer RoR/JS W/M</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Java, Angular, React</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pennylane-sas/fullstack-software-engineer-ror-js-w-m-paris-363056</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2749,34 +2749,34 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>vitaservices GmbH &amp; Co. KG</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>AI-Native Software Engineer (m/w/d)</t>
+          <t>Software Engineer Intern - Financial Services</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, Kubernetes</t>
+          <t>Java, Spring Boot, Angular, React, TypeScript, Kafka, Docker</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-intern-financial-services-paris-450886</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2786,71 +2786,71 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Teampicnic</t>
+          <t>Mirakl - Labs</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Paris, France</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Tech Lead (Java)</t>
+          <t>Software Engineer Apprentice - Connect</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, Kafka, Docker</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/mirakl-labs/software-engineer-apprentice-connect-paris-150457</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>RevenueCat</t>
+          <t>Conflux</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Canada,  Europe,  USA</t>
+          <t>Utrecht, Utrecht, Nederland</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Senior Sales Engineer</t>
+          <t>Senior Java Developer</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, AWS</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/conflux/senior-java-developer-utrecht-224467</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2860,34 +2860,34 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Adikteev</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Remote job</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Staff Site Reliability Engineer</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>AWS</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/adikteev/remote-staff-site-reliability-engineer-paris-357394</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2897,27 +2897,27 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Nebius</t>
+          <t>Accso – Accelerated Solutions GmbH</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Zurich</t>
+          <t>Darmstadt</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
+          <t>Senior Fullstack Entwickler - Java, Spring, Angular*</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Kubernetes</t>
+          <t>Java, Angular, React</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
+          <t>https://www.arbeitnow.com/jobs/companies/accso-accelerated-solutions-gmbh/senior-fullstack-entwickler-java-spring-angular-darmstadt-138755</t>
         </is>
       </c>
     </row>
@@ -2934,27 +2934,27 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>vitaservices GmbH &amp; Co. KG</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Villeneuve-d'Ascq, Nord</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
+          <t>AI-Native Software Engineer (m/w/d)</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>TypeScript, Kafka, Docker, AWS</t>
+          <t>Java, Spring Boot, Angular, Kubernetes</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
+          <t>https://www.arbeitnow.com/jobs/companies/vitaservices-gmbh-co-kg/ai-native-software-engineer-berlin-79664</t>
         </is>
       </c>
     </row>
@@ -2971,108 +2971,108 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Teampicnic</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Lille - Btwin Village, Nord</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
+          <t>Tech Lead (Java)</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Kafka, Kubernetes</t>
+          <t>Java, Spring Boot, TypeScript, Kafka, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/teampicnic/tech-lead-java-amsterdam-378374</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Tavily</t>
+          <t>RevenueCat</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Canada,  Europe,  USA</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
+          <t>Senior Sales Engineer</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Angular, React</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
+          <t>https://jobicy.com/jobs/153225-senior-sales-engineer-2</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Java, React, AWS</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-rendering-engineer-zurich-220466</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -3082,34 +3082,34 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Nebius</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Zurich</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Tech Lead - Platform</t>
+          <t>Senior Software Engineer (Agentic Search) - Web Access Engineer</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes</t>
+          <t>Kubernetes</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
+          <t>https://www.arbeitnow.ch/jobs/companies/nebius/senior-software-engineer-agentic-search-web-access-engineer-zurich-380244</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -3119,34 +3119,34 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Pelico</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Villeneuve-d'Ascq, Nord</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Tech Lead - Solutions</t>
+          <t>Senior Software Engineer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>TypeScript, Kafka, Docker, AWS</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/senior-software-engineer-data-factory-villeneuve-dascq-nord-185021</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -3156,27 +3156,27 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>MILES Mobility</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Lille - Btwin Village, Nord</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
+          <t>Engineering Manager - Sport Process - Worldwide Offer (f/m/d)</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/engineering-manager-sport-process-worldwide-offer-lille-btwin-village-nord-183173</t>
         </is>
       </c>
     </row>
@@ -3193,34 +3193,34 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Keylane</t>
+          <t>Tavily</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Utrecht, Netherlands</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Medior / Senior Java Software Engineer</t>
+          <t>Senior Software Engineer (Agentic Search) – Web Rendering Engineer</t>
         </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Java, Angular, Docker</t>
+          <t>Angular, React</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/tavily/senior-software-engineer-agentic-search-web-rendering-engineer-444896</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -3230,108 +3230,108 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Zone &amp;#038; Co</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>UK</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>GTM Engineer</t>
+          <t>Sr. Software Engineer (Remote Eligible from Bulgaria)</t>
         </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, AWS</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
+          <t>https://jobicy.com/jobs/155172-sr-software-engineer-remote-eligible-from-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Smartsheet</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
+          <t>Tech Lead - Platform</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript, Kubernetes</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-platform-paris-355949</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Five9</t>
+          <t>Pelico</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Frontend</t>
+          <t>Tech Lead - Solutions</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/pelico/tech-lead-solutions-paris-46303</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -3341,17 +3341,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>MILES Mobility</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Senior Data Engineer (x/f/m)</t>
+          <t>Senior React Native Engineer - App Owner (w/m/x/d)</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3361,14 +3361,14 @@
       </c>
       <c r="G79" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
+          <t>https://www.arbeitnow.com/jobs/companies/miles-mobility/senior-react-native-engineer-app-owner-d-berlin-421435</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -3378,27 +3378,27 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Keylane</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Utrecht, Netherlands</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>IA Engineer Intern (x/f/m) - Paris</t>
+          <t>Medior / Senior Java Software Engineer</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Angular, Docker</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
+          <t>https://www.arbeitnow.nl/jobs/companies/keylane/medior-senior-java-software-engineer-utrecht-259177</t>
         </is>
       </c>
     </row>
@@ -3415,27 +3415,27 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>CoderPad</t>
+          <t>Zone &amp;#038; Co</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>UK</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Lead Software Engineer</t>
+          <t>GTM Engineer</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
+          <t>https://jobicy.com/jobs/155142-gtm-engineer-4</t>
         </is>
       </c>
     </row>
@@ -3447,76 +3447,76 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Certivity</t>
+          <t>Smartsheet</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>München - HQ</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
+          <t>Software Engineer (Remote Eligible in Bulgaria)</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
+          <t>https://jobicy.com/jobs/155069-software-engineer-remote-eligible-in-bulgaria</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Valtech</t>
+          <t>Five9</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Portugal</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>FR - Tech Lead Coremedia</t>
+          <t>Senior Software Engineer - Frontend</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
+          <t>https://jobicy.com/jobs/155063-senior-software-engineer-frontend-2</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -3526,34 +3526,34 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Bikeleasing</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Remote Deutschland</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>Senior QA Engineer (gn)</t>
+          <t>Senior Data Engineer (x/f/m)</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-data-engineer-paris-paris-87219</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -3563,71 +3563,71 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Perk</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>Senior PR Manager</t>
+          <t>IA Engineer Intern (x/f/m) - Paris</t>
         </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/ia-engineer-intern-paris-paris-paris-47395</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Arbeitnow</t>
+          <t>Jobicy</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>freiheit.com technologies</t>
+          <t>CoderPad</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Hamburg</t>
+          <t>France</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Hackers wanted – Senior Software Engineer</t>
+          <t>Lead Software Engineer</t>
         </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>Java, Angular, TypeScript</t>
+          <t>Java, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
+          <t>https://jobicy.com/jobs/153066-lead-software-engineer</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -3637,34 +3637,34 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Decathlontechnology</t>
+          <t>Certivity</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>München - HQ</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Full Stack Developer - Data Factory (f/m/d)</t>
+          <t>Python Engineer – Web Crawling &amp; Data Extraction (m/f/d)</t>
         </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
+          <t>Java, Spring Boot, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
+          <t>https://www.arbeitnow.com/jobs/companies/certivity/python-engineer-web-crawling-data-extraction-munchen-hq-492504</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -3674,34 +3674,34 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Fact Finder</t>
+          <t>Valtech</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
+          <t>FR - Tech Lead Coremedia</t>
         </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
+          <t>https://www.arbeitnow.com/jobs/companies/valtech/fr-tech-lead-coremedia-142170</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-10-09</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -3711,34 +3711,34 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>databricks</t>
+          <t>Bikeleasing</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Remote Deutschland</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Forward Deployed Engineer</t>
+          <t>Senior QA Engineer (gn)</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>Java, TypeScript</t>
+          <t>Java, Spring Boot, React, TypeScript, AWS</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
+          <t>https://www.arbeitnow.com/jobs/companies/bikeleasing/remote-senior-qa-engineer-gn-298617</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -3748,34 +3748,34 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>Perk</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>Senior Java Fullstack Developer (m/w/d)</t>
+          <t>Senior PR Manager</t>
         </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/perk/senior-pr-manager-london-482991</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -3785,34 +3785,34 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>virtual7 GmbH</t>
+          <t>freiheit.com technologies</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Hamburg, Hamburg, Deutschland</t>
+          <t>Hamburg</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
+          <t>Hackers wanted – Senior Software Engineer</t>
         </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, Angular, TypeScript</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
+          <t>https://www.arbeitnow.com/jobs/companies/freiheitcom-technologies/hackers-wanted-senior-software-engineer-hamburg-118878</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -3822,34 +3822,34 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Think Cell</t>
+          <t>Decathlontechnology</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
+          <t>Full Stack Developer - Data Factory (f/m/d)</t>
         </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>Java, Spring Boot</t>
+          <t>Java, Angular, React, TypeScript, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/decathlontechnology/full-stack-developer-data-factory-paris-paris-431050</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -3859,34 +3859,34 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>Fact Finder</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>QA Engineer Intern (6 months)</t>
+          <t>Staff Frontend Engineer / Frontend Architect (m/f/d)</t>
         </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>React, TypeScript, Docker, Kubernetes</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
+          <t>https://www.arbeitnow.com/jobs/companies/fact-finder/staff-frontend-engineer-frontend-architect-berlin-122504</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-10-08</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -3896,27 +3896,27 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>shifttechnology</t>
+          <t>databricks</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>London</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>Full stack Engineer Intern (6 months)</t>
+          <t>Forward Deployed Engineer</t>
         </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t>Java, React</t>
+          <t>Java, TypeScript</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/databricks/forward-deployed-engineer-london-285228</t>
         </is>
       </c>
     </row>
@@ -3933,27 +3933,27 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Researchgate</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Senior Frontend Engineer - React</t>
+          <t>Senior Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>React, TypeScript</t>
+          <t>Java, React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-418601</t>
         </is>
       </c>
     </row>
@@ -3970,27 +3970,27 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>orderbird GmbH</t>
+          <t>virtual7 GmbH</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Berlin</t>
+          <t>Hamburg, Hamburg, Deutschland</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Head of Software Engineering (d/f/m)</t>
+          <t>(Senior) Java Fullstack Developer (m/w/d)</t>
         </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>Java, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
+          <t>https://www.arbeitnow.com/jobs/companies/virtual7-gmbh/senior-java-fullstack-developer-hamburg-44621</t>
         </is>
       </c>
     </row>
@@ -4007,27 +4007,27 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Hawkeyeinnovations</t>
+          <t>Think Cell</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Budapest, Hungary</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer - (HawkAI)</t>
+          <t>(Senior) Full Stack Developer - Web (f/m/d)</t>
         </is>
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Docker, AWS</t>
+          <t>Java, Spring Boot</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
+          <t>https://www.arbeitnow.com/jobs/companies/think-cell/senior-full-stack-developer-web-442103</t>
         </is>
       </c>
     </row>
@@ -4044,27 +4044,27 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Python (x/f/m)</t>
+          <t>QA Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
+          <t>React, TypeScript, Docker, Kubernetes</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/qa-engineer-intern-6-months-113722</t>
         </is>
       </c>
     </row>
@@ -4081,27 +4081,27 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>shifttechnology</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>EU Remote</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
+          <t>Full stack Engineer Intern (6 months)</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>Java, React</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/shifttechnology/full-stack-engineer-intern-6-months-327480</t>
         </is>
       </c>
     </row>
@@ -4118,27 +4118,27 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Doctolib</t>
+          <t>Researchgate</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Paris, Paris</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>Design System Director (x/f/m)</t>
+          <t>Senior Frontend Engineer - React</t>
         </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript</t>
+          <t>React, TypeScript</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
+          <t>https://www.arbeitnow.com/jobs/companies/researchgate/senior-frontend-engineer-react-berlin-163857</t>
         </is>
       </c>
     </row>
@@ -4150,32 +4150,32 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Dataiku</t>
+          <t>orderbird GmbH</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+          <t>Berlin</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>Fullstack Software Engineer - Core</t>
+          <t>Head of Software Engineering (d/f/m)</t>
         </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+          <t>Java, React, Docker, Kubernetes, AWS</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+          <t>https://www.arbeitnow.com/jobs/companies/orderbird-gmbh/head-of-software-engineering-berlin-135166</t>
         </is>
       </c>
     </row>
@@ -4192,27 +4192,27 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Baringa</t>
+          <t>Hawkeyeinnovations</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>London</t>
+          <t>Budapest, Hungary</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>Senior Software Engineer - Future Opportunities</t>
+          <t>Senior Full Stack Engineer - (HawkAI)</t>
         </is>
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, Angular, React, AWS</t>
+          <t>Java, React, TypeScript, Docker, AWS</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/hawkeyeinnovations/senior-full-stack-engineer-hawkai-budapest-73855</t>
         </is>
       </c>
     </row>
@@ -4229,143 +4229,328 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>autoscout24</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>EU Remote</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Senior Fullstack Engineer (m/f/d)</t>
+          <t>Senior Software Engineer - Python (x/f/m)</t>
         </is>
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>Java, React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript, Kafka, Kubernetes</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
         <is>
-          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/senior-software-engineer-python-paris-paris-159858</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Sporty Group</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Europe</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>Frontend Engineering Team Lead - MarTech</t>
+          <t>Director of Developer Experience - Platform Engineering (x/f/m)</t>
         </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/director-of-developer-experience-platform-engineering-paris-paris-413651</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-10-07</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Jobicy</t>
+          <t>Arbeitnow</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>infisical</t>
+          <t>Doctolib</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Brazil,  Canada,  Europe,  USA</t>
+          <t>Paris, Paris</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Senior Full Stack Engineer</t>
+          <t>Design System Director (x/f/m)</t>
         </is>
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>React, TypeScript, AWS</t>
+          <t>Java, React, TypeScript</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
         <is>
-          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+          <t>https://www.arbeitnow.fr/jobs/companies/doctolib/design-system-director-paris-paris-264979</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Dataiku</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>France,  Germany,  Netherlands,  Spain,  UK</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Fullstack Software Engineer - Core</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Java, Angular, React, Docker, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/152707-fullstack-software-engineer-core</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Baringa</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>London</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Senior Software Engineer - Future Opportunities</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, Angular, React, AWS</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.co.uk/jobs/companies/baringa/senior-software-engineer-future-opportunities-london-336075</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>autoscout24</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>EU Remote</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Senior Fullstack Engineer (m/f/d)</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Java, React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>https://www.arbeitnow.com/jobs/companies/autoscout24/senior-fullstack-engineer-173116</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
           <t>2026-10-07</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
-        <is>
-          <t>Arbeitnow</t>
-        </is>
-      </c>
-      <c r="C106" t="inlineStr">
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Sporty Group</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>Europe</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Frontend Engineering Team Lead - MarTech</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Java, Spring Boot, TypeScript, Kubernetes, AWS</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/149869-frontend-engineering-team-lead-martech</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Jobicy</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>infisical</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>Brazil,  Canada,  Europe,  USA</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Senior Full Stack Engineer</t>
+        </is>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>React, TypeScript, AWS</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>https://jobicy.com/jobs/154483-senior-full-stack-engineer-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-10-07</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Arbeitnow</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
         <is>
           <t>Eye Security</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr">
+      <c r="D111" t="inlineStr">
         <is>
           <t>Berlin - hybrid</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr">
+      <c r="E111" t="inlineStr">
         <is>
           <t>Senior Software Engineer (m/f/x)</t>
         </is>
       </c>
-      <c r="F106" t="inlineStr">
+      <c r="F111" t="inlineStr">
         <is>
           <t>Java, React, TypeScript</t>
         </is>
       </c>
-      <c r="G106" t="inlineStr">
+      <c r="G111" t="inlineStr">
         <is>
           <t>https://www.arbeitnow.com/jobs/companies/eye-security/senior-software-engineer-berlin-248595</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G106"/>
+  <autoFilter ref="A1:G111"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>